<commit_message>
corte semanal cartera cpel
corte semanal de cartera cpel
</commit_message>
<xml_diff>
--- a/cartera-cpel/data/datos_proyectos.xlsx
+++ b/cartera-cpel/data/datos_proyectos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\CPEL_APP_V1\cartera-cpel\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\proyectos_cpel-claude-code-improvement-analysis-0rbe6x 2\proyectos_cpel-claude-code-improvement-analysis-0rbe6x\cartera-cpel\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77AEE5E2-6E0F-4D00-9CA8-C703BC0F25A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8634B29E-71D4-4818-93A2-4726F296CF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -604,35 +604,6 @@
     <t>240</t>
   </si>
   <si>
-    <t>•	11 y 12 sept: Arribaron 15 contenedores con 15 Centros de Transformación (30 inversores), al almacén temporal del Contratista en Puerto Peñasco. Con este suministro se tiene un total acumulado de 33 CT's de 38 totales en Sitio (86.84%).
-•	11 al 15-sep: Arribaron 17 contenedores con 12,064 Hincas (parte del Sistema de Seguimiento), en la plataforma provisional en sitio. Con este suministro se tiene un total acumulado de 39,649 hincas de 84,182 en Sitio (47.09%).
-•	Continúan actividades de hincado de perfiles correspondientes al Sistema de Seguimiento, en los cuadrantes CT-02 y CT-03, Zona Sur del Polígono, así como actividades de replanteo, conformación de plataformas en Centro de Interconexión con un avance del 70%, así como trabajos de conformación de plataforma en Subestación de Maniobras Puerto Peñasco 400 kV con un avance del 10%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•	Obra civil: Continúan los trabajos limpieza del terreno en la Zona Norte (subzona 4) del polígono de la CFV, con un avance de 73.12 Ha de 465.68 Ha (15.70%). Continúan trabajos de nivelación de terreno con un avance del 40.00 Ha de 465.68 Ha (8.58%).
-•	Ambiental: Continúan los trabajos de rescate y reubicación de flora y fauna dentro del polígono de la CFV Zona Norte (subzonas 1, 2, 3, 4 y 5). </t>
-  </si>
-  <si>
-    <t xml:space="preserve">•	En proceso de formalización del Primer Convenio Modificatorio del Contrato F/1320/001/2022.
-•	Se encuentra en elaboración e integración del Análisis de Viabilidad del P.H. Chicoasén II, para la solicitud de recursos para finalizar la obra.
-•	Obra Civil: Continúa la construcción de la Pantalla Impermeable del eje principal, Empaque de los Tubos de Aspiración de las Unidades de Casa de Máquinas, así como colocación de Hardfill en Muro de Cierre Margen Izquierda y Toma Ecológica; de igual forma la construcción de la cimentación del Cimacio.
-•	Obra Electromecánica: Continúa el montaje de los Tubos de Aspiración y Columnas fijas de las 3 Unidades; así como la Nariz de Bulbo de la U1, en Casa de Máquinas. En Playa de Montaje se continúa el ensamble del Estator de las 3 Unidades y el Rotor de la U1. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">•	22-sep-26: El Contratista deberá disponer y emplear de todos los recursos materiales y humanos para poder concluir el Proyecto en la fecha programada conforme al Convenio 7. La Contratante estará atenta en detectar y señalar las desviaciones al programa para realizar las acciones necesarias para la recuperación de los posibles retrasos, principalmente en las Pruebas de Puesta y Servicio de las dos Unidades Generadoras, y Aceptación de las mismas.
-•	El Contratista debe incrementar la presencia de personal y darles continuidad a los trabajos en el turno nocturno.
-•	La Contratante y Contratistas se están coordinando para dar atención a los temas relacionados con CENACE y Transmisión de CFE para las Pruebas de Puesta en Servicio y Aceptación de las dos Unidades Generadoras. </t>
-  </si>
-  <si>
-    <t>•	Contrato de Obra Electromecánica Principal (Siemens Energy): Proceso de Terminación Anticipada.
-•	Contrato de Auxiliares de Casa de Maquinas (COSEGO Ingeniería): En conciliación de Convenio Modificatorio para dar vigencia al Contrato y realizar el pago del Hito No. 03 (suministro).
-•	Obra Civil: Suspendidas, a cargo del Gobierno del Estado de Sinaloa. Se realizan reuniones entre la SOP y la CFE para la entrega recepción de las Obras Civiles. Se requiere intervención del área interinstitucional de la CFE para agilizar el proceso de cierre administrativo de los contratos civiles por parte del Gobierno de Sinaloa.</t>
-  </si>
-  <si>
-    <t>•	Obra Civil: La CFE y la Secretaría de Obras Públicas del Estado de Sinaloa atienden los compromisos para la entrega de las obras civiles y están a la espera de que la dependencia confirme la fecha para el cierre administrativo y el finiquito de los contratos.
-•	Obra Electromecánica: Conciliar las Razones Fundadas y Explicitas y celebrar con el Contratista Andritz el Primer Convenio Modificatorio del Contrato No. F/10670-021/2024 de la Obra Electromecánica.</t>
-  </si>
-  <si>
     <t>30/12/2028</t>
   </si>
   <si>
@@ -691,6 +662,43 @@
   </si>
   <si>
     <t>Colocación de Órdenes de Compra de equipos electromecánicos del Parque Fotovoltaico</t>
+  </si>
+  <si>
+    <t>•	25-sep: El Fideicomiso realizó el pago del H5 (5%) y el H9 (5%) por un monto total del $29.4 MDD.
+•	26-sep: El Contratista remitió carta invitación a Pruebas FAT de transformador de potencia.
+•	29-sep: Suministro en sitio de 2,688 hincas (parte del Sistema de Seguimiento), alcanzando un acumulado de 52,956 hincas de 84,182 programadas en sitio (62.90% de avance).
+•	Obra electromecánica: Continúan actividades de hincado de perfiles correspondientes al Sistema de Seguimiento en los cuadrantes CT-01, CT-02, CT-03, CT-04 y CT-05 Zona Sur del Polígono. 
+•	Obra civil: Continúan actividades de replanteo, conformación de plataformas en Centro de Interconexión con un avance del 97%, así como trabajos de conformación de plataforma en Subestación de Maniobras Puerto Peñasco 400 kV con un avance del 65%.</t>
+  </si>
+  <si>
+    <t>•	25 al 28 sep: Trabajos de limpieza y nivelación del terreno para el patio de maniobras de S.E. Cucapah Bco. 3. Asimismo, el 28 de septiembre iniciaron los trabajos de conformación de la plataforma correspondiente.
+•	26-sep: El Contratista remitió carta invitación a Pruebas FAT de cuchillas desconectadoras tripolares CM &amp; CMC.
+•	Ambiental: Continúan los trabajos de rescate y reubicación de flora y fauna dentro del polígono de la CFV Zona Norte (subzonas 1, 2, 3, 4 y 5).
+•	Obra civil: Continúan los trabajos de limpieza del terreno en la Zona Norte (subzona 4) del polígono de la CFV, con un avance de 146.68 Ha de 465.68 Ha (31.49%). Continúan trabajos de nivelación de terreno con un avance de 43.43 Ha de 465.68 Ha (9.32%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•	Se continua con la elaboración e integración del Análisis de Viabilidad del P.H. Chicoasén II, para la solicitud de recursos para finalizar la obra.
+•	25-sep: El Fideicomiso y el Proveedor GE formalizaron el Primer Convenio Modificatorio al Contrato de Adquisiciones de Bienes y prestaciones No. F/1320/001/2022. 
+•	28 y 29-sep: Traslado de los 4 segmentos del Cono Fijo U1 desde el Almacén 205 MI a la plataforma 183 (zona de obras) para iniciar su preensamble. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">•	Continúan las actividades de montaje de equipos y sistemas electromecánicos para la puesta en marcha y entrada en operación de las unidades U1 y U2, programadas para octubre y noviembre de 2026.
+•	En proceso de conciliación los avances parciales de los hitos de suministro de las unidades U1 y U2 (H4 e H5).
+•	Se requiere reforzar los frentes de obra electromecánica y puesta en servicio, así como mantener la continuidad de los trabajos en turno nocturno para mitigar riesgos al programa de ejecución. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">•	Se está gestionando la entrega-recepción de las obras civiles y el cierre del Convenio de Colaboración entre la CFE y el Estado de Sinaloa.
+•	En proceso de conciliación la Terminación Anticipada del Contrato de Obra Electromecánica Principal con SIEMES.
+•	Se esta conciliando el Convenio Modificatorio con el Contratista COSEGO.
+•	Se ha analizado y está pendiente definir si es conveniente realizar la Terminación Anticipada de los Contratos Electromecánicos Auxiliares, dada la Terminación del Contrato de Obra Electromecánica Principal.
+•	Definición del mecanismo de financiamiento para la contratación y culminación de las obras civiles y electromecánicas.
+•	Se ha integrado el paquete técnico de la obra civil y está pendiente el de la electromecánica restante de ejecutar. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">•	Continúa pendiente la contratación de las obras civiles para la conclusión del proyecto.
+•	Se está gestionando la entrega recepción de las obras civiles, así como del finiquito los contratos a cargo de la SOP.
+•	En proceso de gestión, la formalización del Primer Convenio Modificatorio del Contrato No. F/10670-021/2024 de la obra electromecánica con Andritz.
+•	Las condiciones de inseguridad en la zona de influencia del proyecto continúan representando un factor de riesgo para su ejecución. </t>
   </si>
 </sst>
 </file>
@@ -1029,7 +1037,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1076,6 +1084,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1663,28 +1673,28 @@
         <v>70</v>
       </c>
       <c r="F2" s="7">
-        <v>30.76</v>
+        <v>31.46</v>
       </c>
       <c r="G2" s="7">
-        <v>27.79</v>
+        <v>28.48</v>
       </c>
       <c r="H2" s="7">
-        <v>6.05</v>
+        <v>6.18</v>
       </c>
       <c r="I2" s="7">
-        <v>5.29</v>
+        <v>5.48</v>
       </c>
       <c r="J2" s="7">
-        <v>16.350000000000001</v>
+        <v>16.59</v>
       </c>
       <c r="K2" s="7">
-        <v>16.34</v>
+        <v>16.57</v>
       </c>
       <c r="L2" s="7">
-        <v>8.36</v>
+        <v>8.69</v>
       </c>
       <c r="M2" s="7">
-        <v>6.16</v>
+        <v>6.43</v>
       </c>
       <c r="N2" s="7">
         <v>0</v>
@@ -1696,52 +1706,52 @@
         <v>6</v>
       </c>
       <c r="Q2" s="8" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="R2" s="32" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="S2" s="7" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="T2" s="7">
         <v>5</v>
       </c>
       <c r="U2" s="8" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="V2" s="8" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="W2" s="7" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="X2" s="7">
         <v>9</v>
       </c>
       <c r="Y2" s="8" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="Z2" s="8" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="AA2" s="7" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="AB2" s="7">
         <v>8</v>
       </c>
       <c r="AC2" s="8" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="AD2" s="8" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="AE2" s="28" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="AF2" s="9" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="AG2" s="10" t="s">
         <v>71</v>
@@ -1844,10 +1854,10 @@
         <v>94</v>
       </c>
       <c r="F3" s="1">
-        <v>4.76</v>
+        <v>5.26</v>
       </c>
       <c r="G3" s="1">
-        <v>4.08</v>
+        <v>7.59</v>
       </c>
       <c r="H3" s="1">
         <v>2.83</v>
@@ -1856,13 +1866,13 @@
         <v>3.12</v>
       </c>
       <c r="J3" s="1">
-        <v>1.59</v>
+        <v>1.9</v>
       </c>
       <c r="K3" s="1">
-        <v>0.39</v>
+        <v>3.9</v>
       </c>
       <c r="L3" s="1">
-        <v>0.38</v>
+        <v>0.53</v>
       </c>
       <c r="M3" s="1">
         <v>0.56999999999999995</v>
@@ -1877,52 +1887,52 @@
         <v>2</v>
       </c>
       <c r="Q3" s="30" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="R3" s="29" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="S3" s="31" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="T3" s="1">
         <v>3</v>
       </c>
       <c r="U3" s="30" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="V3" s="29" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="W3" s="31" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="X3" s="1">
         <v>5</v>
       </c>
       <c r="Y3" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="Z3" s="29" t="s">
         <v>199</v>
       </c>
-      <c r="Z3" s="29" t="s">
-        <v>205</v>
-      </c>
       <c r="AA3" s="1" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="AB3" s="1">
         <v>4</v>
       </c>
       <c r="AC3" s="30" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="AD3" s="29" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
+      </c>
+      <c r="AF3" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AG3" s="13" t="s">
         <v>71</v>
@@ -2025,34 +2035,34 @@
         <v>112</v>
       </c>
       <c r="F4" s="1">
-        <v>77.44</v>
+        <v>78.510000000000005</v>
       </c>
       <c r="G4" s="1">
-        <v>80.72</v>
+        <v>81.63</v>
       </c>
       <c r="H4" s="1">
         <v>100</v>
       </c>
       <c r="I4" s="1">
-        <v>99.19</v>
+        <v>99.39</v>
       </c>
       <c r="J4" s="1">
-        <v>98.53</v>
+        <v>99.74</v>
       </c>
       <c r="K4" s="1">
-        <v>99.89</v>
+        <v>99.93</v>
       </c>
       <c r="L4" s="1">
-        <v>82.49</v>
+        <v>82.58</v>
       </c>
       <c r="M4" s="1">
-        <v>91.98</v>
+        <v>92.32</v>
       </c>
       <c r="N4" s="1">
-        <v>10.42</v>
+        <v>13.49</v>
       </c>
       <c r="O4" s="1">
-        <v>2.8</v>
+        <v>4.12</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -2070,8 +2080,8 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
       <c r="AE4" s="1"/>
-      <c r="AF4" s="1" t="s">
-        <v>186</v>
+      <c r="AF4" s="34" t="s">
+        <v>206</v>
       </c>
       <c r="AG4" s="13" t="s">
         <v>113</v>
@@ -2169,7 +2179,7 @@
         <v>93.31</v>
       </c>
       <c r="G5" s="1">
-        <v>70.3</v>
+        <v>70.02</v>
       </c>
       <c r="H5" s="1">
         <v>100</v>
@@ -2190,7 +2200,7 @@
         <v>63.5</v>
       </c>
       <c r="N5" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O5" s="1">
         <v>0</v>
@@ -2211,8 +2221,8 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
-      <c r="AF5" s="1" t="s">
-        <v>187</v>
+      <c r="AF5" s="34" t="s">
+        <v>207</v>
       </c>
       <c r="AG5" s="13" t="s">
         <v>122</v>
@@ -2310,13 +2320,13 @@
         <v>100</v>
       </c>
       <c r="G6" s="1">
-        <v>33.43</v>
+        <v>33.64</v>
       </c>
       <c r="H6" s="1">
         <v>100</v>
       </c>
       <c r="I6" s="1">
-        <v>64.92</v>
+        <v>65</v>
       </c>
       <c r="J6" s="1">
         <v>100</v>
@@ -2352,8 +2362,8 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
       <c r="AE6" s="1"/>
-      <c r="AF6" s="1" t="s">
-        <v>188</v>
+      <c r="AF6" s="34" t="s">
+        <v>208</v>
       </c>
       <c r="AG6" s="13" t="s">
         <v>132</v>
@@ -2448,34 +2458,34 @@
         <v>142</v>
       </c>
       <c r="F7" s="2">
-        <v>49.7</v>
+        <v>49.2</v>
       </c>
       <c r="G7" s="2">
-        <v>49.7</v>
+        <v>49.3</v>
       </c>
       <c r="H7" s="2">
-        <v>72.69</v>
+        <v>75.77</v>
       </c>
       <c r="I7" s="2">
-        <v>58.9</v>
+        <v>59.09</v>
       </c>
       <c r="J7" s="2">
-        <v>54.53</v>
+        <v>54.33</v>
       </c>
       <c r="K7" s="2">
-        <v>55.68</v>
+        <v>54.41</v>
       </c>
       <c r="L7" s="2">
-        <v>51.26</v>
+        <v>45.35</v>
       </c>
       <c r="M7" s="2">
-        <v>49.9</v>
+        <v>46.36</v>
       </c>
       <c r="N7" s="2">
-        <v>35.479999999999997</v>
+        <v>14.61</v>
       </c>
       <c r="O7" s="2">
-        <v>0.59</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
@@ -2493,8 +2503,8 @@
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
-      <c r="AF7" s="2" t="s">
-        <v>185</v>
+      <c r="AF7" s="35" t="s">
+        <v>205</v>
       </c>
       <c r="AG7" s="17" t="s">
         <v>143</v>
@@ -2522,7 +2532,7 @@
         <v>147</v>
       </c>
       <c r="AP7" s="19" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="AQ7" s="17"/>
       <c r="AR7" s="17"/>

</xml_diff>

<commit_message>
Cartera CPEL: avance financiero junto al físico en Avance General
- Excel nuevo de datos_proyectos con avanfinProg y avanfinReal.
- La tarjeta "Avance General" se divide: Físico a la izquierda y
  Financiero a la derecha, cada uno con Programado, Real, semáforo
  (texto corto: "Atraso de 13.00 pts") y cambio desde el corte anterior.
  Sin datos financieros se ve como antes, a todo lo ancho.
- El historial guarda finProg/finReal para el cambio semanal del
  financiero (aparece desde el segundo corte que lo tenga).
- La Action "Datos" valida avanfinProg/avanfinReal como porcentajes
  (opcionales).
- Pruebas unitarias y e2e; README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-cpel/data/datos_proyectos.xlsx
+++ b/cartera-cpel/data/datos_proyectos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261A08FB-9AAF-4F64-B6DC-DA18C87F3602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D98CBF-344F-4D5D-AC1E-EB895AB5BCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AZ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$BB$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="178">
   <si>
     <t>id</t>
   </si>
@@ -594,6 +594,12 @@
   </si>
   <si>
     <t>data/VIDEOS/CHICOASEN.mp4</t>
+  </si>
+  <si>
+    <t>avanfinReal</t>
+  </si>
+  <si>
+    <t>avanfinProg</t>
   </si>
 </sst>
 </file>
@@ -880,7 +886,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
@@ -920,8 +926,6 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1227,7 +1231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AZ7"/>
+  <dimension ref="A1:BB7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -1238,43 +1242,44 @@
     <col min="6" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="47.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="17" bestFit="1" customWidth="1"/>
-    <col min="42" max="48" width="16" bestFit="1" customWidth="1"/>
-    <col min="49" max="52" width="16" customWidth="1"/>
+    <col min="9" max="10" width="15.5703125" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="47.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="17" bestFit="1" customWidth="1"/>
+    <col min="44" max="50" width="16" bestFit="1" customWidth="1"/>
+    <col min="51" max="54" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1300,139 +1305,145 @@
         <v>6</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AN1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AM1" s="5" t="s">
+      <c r="AO1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AN1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AO1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AR1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AS1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AT1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AS1" s="5" t="s">
+      <c r="AU1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AT1" s="5" t="s">
+      <c r="AV1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AW1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="AV1" s="5" t="s">
+      <c r="AX1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AW1" s="5" t="s">
+      <c r="AY1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AX1" s="5" t="s">
+      <c r="AZ1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AY1" s="5" t="s">
+      <c r="BA1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AZ1" s="6" t="s">
+      <c r="BB1" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A2" s="24">
         <v>1</v>
       </c>
@@ -1456,106 +1467,110 @@
         <v>32.17</v>
       </c>
       <c r="I2" s="7">
+        <v>53</v>
+      </c>
+      <c r="J2" s="7">
+        <v>40</v>
+      </c>
+      <c r="K2" s="7">
         <v>6.36</v>
       </c>
-      <c r="J2" s="7">
+      <c r="L2" s="7">
         <v>6.46</v>
       </c>
-      <c r="K2" s="7">
+      <c r="M2" s="7">
         <v>19.440000000000001</v>
       </c>
-      <c r="L2" s="7">
+      <c r="N2" s="7">
         <v>17.86</v>
       </c>
-      <c r="M2" s="7">
+      <c r="O2" s="7">
         <v>10.28</v>
       </c>
-      <c r="N2" s="7">
+      <c r="P2" s="7">
         <v>7.85</v>
       </c>
-      <c r="O2" s="7">
+      <c r="Q2" s="7">
         <v>0</v>
       </c>
-      <c r="P2" s="7">
+      <c r="R2" s="7">
         <v>0</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="T2" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="U2" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="V2" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="U2" s="9">
+      <c r="W2" s="9">
         <v>728</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="X2" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="W2" s="10" t="s">
+      <c r="Y2" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="X2" s="10" t="s">
+      <c r="Z2" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="Y2" s="10" t="s">
+      <c r="AA2" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="Z2" s="10" t="s">
+      <c r="AB2" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="AA2" s="10" t="s">
+      <c r="AC2" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="AB2" s="10" t="s">
+      <c r="AD2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="AC2" s="10" t="s">
+      <c r="AE2" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AD2" s="10" t="s">
+      <c r="AF2" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="AE2" s="10" t="s">
+      <c r="AG2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AF2" s="10" t="s">
+      <c r="AH2" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="AG2" s="10" t="s">
+      <c r="AI2" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="AH2" s="9" t="s">
+      <c r="AJ2" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AI2" s="10" t="s">
+      <c r="AK2" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="AJ2" s="10" t="s">
+      <c r="AL2" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="AK2" s="10" t="s">
+      <c r="AM2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="AL2" s="10" t="s">
+      <c r="AN2" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="AM2" s="9" t="s">
+      <c r="AO2" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="AN2" s="9" t="s">
+      <c r="AP2" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="AO2" s="9" t="s">
+      <c r="AQ2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="AP2" s="10"/>
-      <c r="AQ2" s="10"/>
       <c r="AR2" s="10"/>
       <c r="AS2" s="10"/>
       <c r="AT2" s="10"/>
@@ -1564,9 +1579,11 @@
       <c r="AW2" s="10"/>
       <c r="AX2" s="10"/>
       <c r="AY2" s="10"/>
-      <c r="AZ2" s="11"/>
+      <c r="AZ2" s="10"/>
+      <c r="BA2" s="10"/>
+      <c r="BB2" s="11"/>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A3" s="25">
         <v>2</v>
       </c>
@@ -1590,106 +1607,110 @@
         <v>9.6300000000000008</v>
       </c>
       <c r="I3" s="1">
+        <v>30</v>
+      </c>
+      <c r="J3" s="1">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1">
         <v>2.87</v>
       </c>
-      <c r="J3" s="1">
+      <c r="L3" s="1">
         <v>3.21</v>
       </c>
-      <c r="K3" s="1">
+      <c r="M3" s="1">
         <v>5.97</v>
       </c>
-      <c r="L3" s="1">
+      <c r="N3" s="1">
         <v>5.37</v>
       </c>
-      <c r="M3" s="1">
+      <c r="O3" s="1">
         <v>0.91</v>
       </c>
-      <c r="N3" s="1">
+      <c r="P3" s="1">
         <v>1.05</v>
       </c>
-      <c r="O3" s="1">
+      <c r="Q3" s="1">
         <v>0</v>
       </c>
-      <c r="P3" s="1">
+      <c r="R3" s="1">
         <v>0</v>
       </c>
-      <c r="Q3" s="27" t="s">
+      <c r="S3" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="T3" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="U3" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="V3" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="U3" s="12">
+      <c r="W3" s="12">
         <v>730</v>
       </c>
-      <c r="V3" s="12" t="s">
+      <c r="X3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="W3" s="13" t="s">
+      <c r="Y3" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="X3" s="13" t="s">
+      <c r="Z3" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="Y3" s="13" t="s">
+      <c r="AA3" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="Z3" s="13" t="s">
+      <c r="AB3" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="AA3" s="13" t="s">
+      <c r="AC3" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="AB3" s="13" t="s">
+      <c r="AD3" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="AC3" s="13" t="s">
+      <c r="AE3" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="AD3" s="13" t="s">
+      <c r="AF3" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="AE3" s="13" t="s">
+      <c r="AG3" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="AF3" s="13" t="s">
+      <c r="AH3" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="AG3" s="13" t="s">
+      <c r="AI3" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="AH3" s="12" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="AI3" s="13" t="s">
+      <c r="AK3" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="AJ3" s="13" t="s">
+      <c r="AL3" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="AK3" s="13" t="s">
+      <c r="AM3" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="AL3" s="13" t="s">
+      <c r="AN3" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="AM3" s="12" t="s">
+      <c r="AO3" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="AN3" s="12" t="s">
+      <c r="AP3" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="AO3" s="12" t="s">
+      <c r="AQ3" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="AP3" s="13"/>
-      <c r="AQ3" s="13"/>
       <c r="AR3" s="13"/>
       <c r="AS3" s="13"/>
       <c r="AT3" s="13"/>
@@ -1698,9 +1719,11 @@
       <c r="AW3" s="13"/>
       <c r="AX3" s="13"/>
       <c r="AY3" s="13"/>
-      <c r="AZ3" s="14"/>
+      <c r="AZ3" s="13"/>
+      <c r="BA3" s="13"/>
+      <c r="BB3" s="14"/>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A4" s="25">
         <v>3</v>
       </c>
@@ -1724,62 +1747,66 @@
         <v>84.36</v>
       </c>
       <c r="I4" s="1">
-        <v>100</v>
+        <v>81.39</v>
       </c>
       <c r="J4" s="1">
-        <v>99.63</v>
+        <v>72.08</v>
       </c>
       <c r="K4" s="1">
         <v>100</v>
       </c>
       <c r="L4" s="1">
+        <v>99.63</v>
+      </c>
+      <c r="M4" s="1">
         <v>100</v>
       </c>
-      <c r="M4" s="1">
+      <c r="N4" s="1">
+        <v>100</v>
+      </c>
+      <c r="O4" s="1">
         <v>83.08</v>
       </c>
-      <c r="N4" s="1">
+      <c r="P4" s="1">
         <v>92.58</v>
       </c>
-      <c r="O4" s="1">
+      <c r="Q4" s="1">
         <v>25.84</v>
       </c>
-      <c r="P4" s="1">
+      <c r="R4" s="1">
         <v>15.41</v>
       </c>
-      <c r="Q4" s="27" t="s">
+      <c r="S4" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="U4" s="15">
+      <c r="W4" s="15">
         <v>1420</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="W4" s="12"/>
-      <c r="X4" s="13" t="s">
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="Y4" s="13" t="s">
+      <c r="AA4" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="Z4" s="13" t="s">
+      <c r="AB4" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="AA4" s="13" t="s">
+      <c r="AC4" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="AB4" s="12"/>
-      <c r="AC4" s="12"/>
       <c r="AD4" s="12"/>
       <c r="AE4" s="12"/>
       <c r="AF4" s="12"/>
@@ -1792,41 +1819,43 @@
       <c r="AM4" s="12"/>
       <c r="AN4" s="12"/>
       <c r="AO4" s="12"/>
-      <c r="AP4" s="13" t="s">
+      <c r="AP4" s="12"/>
+      <c r="AQ4" s="12"/>
+      <c r="AR4" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="AQ4" s="13" t="s">
+      <c r="AS4" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="AR4" s="13" t="s">
+      <c r="AT4" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="AS4" s="13" t="s">
+      <c r="AU4" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="AT4" s="13" t="s">
+      <c r="AV4" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="AU4" s="13" t="s">
+      <c r="AW4" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="AV4" s="13" t="s">
+      <c r="AX4" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="AW4" s="13" t="s">
+      <c r="AY4" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="AX4" s="13" t="s">
+      <c r="AZ4" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="AY4" s="13" t="s">
+      <c r="BA4" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="AZ4" s="14" t="s">
+      <c r="BB4" s="14" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A5" s="25">
         <v>4</v>
       </c>
@@ -1850,62 +1879,66 @@
         <v>74.47</v>
       </c>
       <c r="I5" s="1">
-        <v>100</v>
+        <v>63.79</v>
       </c>
       <c r="J5" s="1">
-        <v>100</v>
+        <v>62.56</v>
       </c>
       <c r="K5" s="1">
         <v>100</v>
       </c>
       <c r="L5" s="1">
+        <v>100</v>
+      </c>
+      <c r="M5" s="1">
+        <v>100</v>
+      </c>
+      <c r="N5" s="1">
         <v>93.19</v>
       </c>
-      <c r="M5" s="1">
+      <c r="O5" s="1">
         <v>93.37</v>
       </c>
-      <c r="N5" s="1">
+      <c r="P5" s="1">
         <v>63.5</v>
       </c>
-      <c r="O5" s="1">
+      <c r="Q5" s="1">
         <v>0</v>
       </c>
-      <c r="P5" s="1">
+      <c r="R5" s="1">
         <v>0</v>
       </c>
-      <c r="Q5" s="27" t="s">
+      <c r="S5" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="R5" s="12" t="s">
+      <c r="T5" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="S5" s="12" t="s">
+      <c r="U5" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="T5" s="12" t="s">
+      <c r="V5" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="U5" s="15">
+      <c r="W5" s="15">
         <v>1720</v>
       </c>
-      <c r="V5" s="12" t="s">
+      <c r="X5" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="W5" s="12"/>
-      <c r="X5" s="13" t="s">
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="Y5" s="13" t="s">
+      <c r="AA5" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="Z5" s="13" t="s">
+      <c r="AB5" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="AA5" s="13" t="s">
+      <c r="AC5" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="AB5" s="12"/>
-      <c r="AC5" s="12"/>
       <c r="AD5" s="12"/>
       <c r="AE5" s="12"/>
       <c r="AF5" s="12"/>
@@ -1918,41 +1951,43 @@
       <c r="AM5" s="12"/>
       <c r="AN5" s="12"/>
       <c r="AO5" s="12"/>
-      <c r="AP5" s="13" t="s">
+      <c r="AP5" s="12"/>
+      <c r="AQ5" s="12"/>
+      <c r="AR5" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="AQ5" s="13" t="s">
+      <c r="AS5" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="AR5" s="13" t="s">
+      <c r="AT5" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="AS5" s="13" t="s">
+      <c r="AU5" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="AT5" s="13" t="s">
+      <c r="AV5" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="AU5" s="13" t="s">
+      <c r="AW5" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="AV5" s="13" t="s">
+      <c r="AX5" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="AW5" s="13" t="s">
+      <c r="AY5" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="AX5" s="13" t="s">
+      <c r="AZ5" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="AY5" s="13" t="s">
+      <c r="BA5" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="AZ5" s="14" t="s">
+      <c r="BB5" s="14" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A6" s="25">
         <v>5</v>
       </c>
@@ -1979,59 +2014,63 @@
         <v>100</v>
       </c>
       <c r="J6" s="1">
-        <v>64.92</v>
+        <v>24</v>
       </c>
       <c r="K6" s="1">
         <v>100</v>
       </c>
       <c r="L6" s="1">
-        <v>45.2</v>
+        <v>64.92</v>
       </c>
       <c r="M6" s="1">
         <v>100</v>
       </c>
       <c r="N6" s="1">
-        <v>12.53</v>
+        <v>45.2</v>
       </c>
       <c r="O6" s="1">
         <v>100</v>
       </c>
       <c r="P6" s="1">
+        <v>12.53</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>100</v>
+      </c>
+      <c r="R6" s="1">
         <v>0</v>
       </c>
-      <c r="Q6" s="27" t="s">
+      <c r="S6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="R6" s="12" t="s">
+      <c r="T6" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="S6" s="12" t="s">
+      <c r="U6" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="T6" s="12" t="s">
+      <c r="V6" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="U6" s="15">
+      <c r="W6" s="15">
         <v>1896</v>
       </c>
-      <c r="V6" s="12" t="s">
+      <c r="X6" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="W6" s="12"/>
-      <c r="X6" s="13" t="s">
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="Y6" s="13" t="s">
+      <c r="AA6" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="Z6" s="13" t="s">
+      <c r="AB6" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="AA6" s="13" t="s">
+      <c r="AC6" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="AB6" s="12"/>
-      <c r="AC6" s="12"/>
       <c r="AD6" s="12"/>
       <c r="AE6" s="12"/>
       <c r="AF6" s="12"/>
@@ -2044,41 +2083,43 @@
       <c r="AM6" s="12"/>
       <c r="AN6" s="12"/>
       <c r="AO6" s="12"/>
-      <c r="AP6" s="13">
+      <c r="AP6" s="12"/>
+      <c r="AQ6" s="12"/>
+      <c r="AR6" s="13">
         <v>10</v>
       </c>
-      <c r="AQ6" s="13">
+      <c r="AS6" s="13">
         <v>46.85</v>
       </c>
-      <c r="AR6" s="13">
+      <c r="AT6" s="13">
         <v>54.5</v>
       </c>
-      <c r="AS6" s="13">
+      <c r="AU6" s="13">
         <v>2</v>
       </c>
-      <c r="AT6" s="13" t="s">
+      <c r="AV6" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="AU6" s="13">
+      <c r="AW6" s="13">
         <v>11.5</v>
       </c>
-      <c r="AV6" s="13">
+      <c r="AX6" s="13">
         <v>50</v>
       </c>
-      <c r="AW6" s="13" t="s">
+      <c r="AY6" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="AX6" s="13">
+      <c r="AZ6" s="13">
         <v>31.48</v>
       </c>
-      <c r="AY6" s="13">
+      <c r="BA6" s="13">
         <v>21.193000000000001</v>
       </c>
-      <c r="AZ6" s="14">
+      <c r="BB6" s="14">
         <v>8944</v>
       </c>
     </row>
-    <row r="7" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26">
         <v>6</v>
       </c>
@@ -2104,62 +2145,66 @@
         <v>51.68</v>
       </c>
       <c r="I7" s="2">
+        <v>54.57</v>
+      </c>
+      <c r="J7" s="2">
+        <v>53.51</v>
+      </c>
+      <c r="K7" s="2">
         <v>79.56</v>
       </c>
-      <c r="J7" s="2">
+      <c r="L7" s="2">
         <v>59.42</v>
       </c>
-      <c r="K7" s="2">
+      <c r="M7" s="2">
         <v>56.6</v>
       </c>
-      <c r="L7" s="2">
+      <c r="N7" s="2">
         <v>57.05</v>
       </c>
-      <c r="M7" s="2">
+      <c r="O7" s="2">
         <v>47.71</v>
       </c>
-      <c r="N7" s="2">
+      <c r="P7" s="2">
         <v>47.4</v>
       </c>
-      <c r="O7" s="2">
+      <c r="Q7" s="2">
         <v>18.07</v>
       </c>
-      <c r="P7" s="2">
+      <c r="R7" s="2">
         <v>0.56000000000000005</v>
       </c>
-      <c r="Q7" s="28" t="s">
+      <c r="S7" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="R7" s="16" t="s">
+      <c r="T7" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="S7" s="16" t="s">
+      <c r="U7" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="T7" s="16" t="s">
+      <c r="V7" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="U7" s="17">
+      <c r="W7" s="17">
         <v>1750</v>
       </c>
-      <c r="V7" s="16" t="s">
+      <c r="X7" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="W7" s="16"/>
-      <c r="X7" s="18" t="s">
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="Y7" s="18" t="s">
+      <c r="AA7" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="Z7" s="18" t="s">
+      <c r="AB7" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="AA7" s="18" t="s">
+      <c r="AC7" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="AB7" s="16"/>
-      <c r="AC7" s="16"/>
       <c r="AD7" s="16"/>
       <c r="AE7" s="16"/>
       <c r="AF7" s="16"/>
@@ -2172,42 +2217,44 @@
       <c r="AM7" s="16"/>
       <c r="AN7" s="16"/>
       <c r="AO7" s="16"/>
-      <c r="AP7" s="18" t="s">
+      <c r="AP7" s="16"/>
+      <c r="AQ7" s="16"/>
+      <c r="AR7" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="AQ7" s="18" t="s">
+      <c r="AS7" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="AR7" s="18" t="s">
+      <c r="AT7" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="AS7" s="18" t="s">
+      <c r="AU7" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="AT7" s="18" t="s">
+      <c r="AV7" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="AU7" s="18" t="s">
+      <c r="AW7" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="AV7" s="18" t="s">
+      <c r="AX7" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AW7" s="18" t="s">
+      <c r="AY7" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="AX7" s="18" t="s">
+      <c r="AZ7" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="AY7" s="18" t="s">
+      <c r="BA7" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="AZ7" s="19" t="s">
+      <c r="BB7" s="19" t="s">
         <v>152</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:BB1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>